<commit_message>
Fixed errors and added new updates
</commit_message>
<xml_diff>
--- a/testData/LoginData.xlsx
+++ b/testData/LoginData.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29910"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30128"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2B302B38-C610-4DE4-8168-9CCF9C286BE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EE585B15-937E-499A-B567-9280D28BFF68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,42 +31,85 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="12">
-  <si>
-    <t>username</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="22">
+  <si>
+    <t>email</t>
   </si>
   <si>
     <t>password</t>
   </si>
   <si>
-    <t>res</t>
+    <t>expected result</t>
+  </si>
+  <si>
+    <t>scenario</t>
+  </si>
+  <si>
+    <t>greenmikey@gmail.com</t>
+  </si>
+  <si>
+    <t>valid</t>
+  </si>
+  <si>
+    <t>valid login</t>
+  </si>
+  <si>
+    <t>maya246@gmail.com</t>
+  </si>
+  <si>
+    <t>invalid</t>
+  </si>
+  <si>
+    <t>wrong password</t>
+  </si>
+  <si>
+    <t>chris789@gmail.com</t>
+  </si>
+  <si>
+    <t>wrong email</t>
+  </si>
+  <si>
+    <t>abc123@gmail.com</t>
+  </si>
+  <si>
+    <t>test@123</t>
+  </si>
+  <si>
+    <t>wrong email and password</t>
+  </si>
+  <si>
+    <r>
+      <t>Jane</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="1"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>#25</t>
+    </r>
+  </si>
+  <si>
+    <t>missing email</t>
   </si>
   <si>
     <t>janedoe25@gmail.com</t>
   </si>
   <si>
-    <t>Ef@067074</t>
-  </si>
-  <si>
-    <t>valid</t>
-  </si>
-  <si>
-    <t>maya@gmail.com</t>
-  </si>
-  <si>
-    <t>invalid</t>
-  </si>
-  <si>
-    <t>mike@gmail.com</t>
-  </si>
-  <si>
-    <t>april@gmail.com</t>
-  </si>
-  <si>
-    <t>abc123@gmail.com</t>
-  </si>
-  <si>
-    <t>test@123</t>
+    <t>missing password</t>
+  </si>
+  <si>
+    <t>both empty</t>
+  </si>
+  <si>
+    <t>invalidemail</t>
+  </si>
+  <si>
+    <t>invalid email format</t>
   </si>
 </sst>
 </file>
@@ -82,19 +125,19 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
+      <b/>
       <sz val="11"/>
-      <color theme="10"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <charset val="1"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -121,18 +164,22 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -445,86 +492,139 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="28.85546875" customWidth="1"/>
     <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="24.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" s="2" customFormat="1">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:4" s="1" customFormat="1">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3">
-      <c r="A2" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" t="s">
+    </row>
+    <row r="2" spans="1:4">
+      <c r="A2" s="4" t="s">
         <v>4</v>
+      </c>
+      <c r="B2" s="5">
+        <v>123456</v>
       </c>
       <c r="C2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="3" spans="1:3">
-      <c r="A3" s="1" t="s">
+      <c r="D2" t="s">
         <v>6</v>
       </c>
-      <c r="B3">
-        <v>12345</v>
+    </row>
+    <row r="3" spans="1:4">
+      <c r="A3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="5">
+        <v>2468</v>
       </c>
       <c r="C3" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3">
-      <c r="A4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B4">
-        <v>2468</v>
+      <c r="D3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4">
+      <c r="A4" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="5">
+        <v>54321</v>
       </c>
       <c r="C4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3">
-      <c r="A5" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B5">
-        <v>54321</v>
+        <v>8</v>
+      </c>
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4">
+      <c r="A5" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>13</v>
       </c>
       <c r="C5" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3">
-      <c r="A6" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" t="s">
-        <v>11</v>
+        <v>8</v>
+      </c>
+      <c r="D5" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4">
+      <c r="A6" s="4"/>
+      <c r="B6" s="4" t="s">
+        <v>15</v>
       </c>
       <c r="C6" t="s">
-        <v>7</v>
+        <v>8</v>
+      </c>
+      <c r="D6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4">
+      <c r="A7" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="3"/>
+      <c r="C7" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4">
+      <c r="B8" s="3"/>
+      <c r="C8" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4">
+      <c r="A9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="A2" r:id="rId1" xr:uid="{3DFB39DA-B85D-4393-83CB-3E6982DEEE18}"/>
-    <hyperlink ref="A3" r:id="rId2" xr:uid="{730836E7-F9D6-444C-8BF6-72B45A6905CB}"/>
-    <hyperlink ref="A4" r:id="rId3" xr:uid="{7135546F-A208-40E2-BB33-380ECDB8AEFA}"/>
-    <hyperlink ref="A5" r:id="rId4" xr:uid="{3972A25D-1BF2-4F8A-A319-FB4EF83F21DD}"/>
-    <hyperlink ref="A6" r:id="rId5" xr:uid="{89DE4BD1-AC45-451A-9BDF-8AF0AB5B6FB8}"/>
+    <hyperlink ref="A4" r:id="rId1" xr:uid="{3972A25D-1BF2-4F8A-A319-FB4EF83F21DD}"/>
+    <hyperlink ref="A5" r:id="rId2" xr:uid="{89DE4BD1-AC45-451A-9BDF-8AF0AB5B6FB8}"/>
+    <hyperlink ref="A7" r:id="rId3" xr:uid="{18B85BDA-7969-4C3B-8287-A2AC85EDAA2A}"/>
+    <hyperlink ref="A3" r:id="rId4" xr:uid="{7135546F-A208-40E2-BB33-380ECDB8AEFA}"/>
+    <hyperlink ref="A2" r:id="rId5" xr:uid="{3DFB39DA-B85D-4393-83CB-3E6982DEEE18}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>